<commit_message>
Add Publisher IPI 01372389230 to the Publisher cue rows
Column P (Publisher IPI #, hidden in the template) now holds
01372389230 on rows 21/23/25/27/29/31, stored as text so the leading
zero survives the column's numeric format. BMI account 4380631 is
recorded in the review notes -- the template has no field for it.
QC re-run: 57 checks, all pass.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Cue_Sheet_The_Dark_Awaits_COMPLETED.xlsx
+++ b/Cue_Sheet_The_Dark_Awaits_COMPLETED.xlsx
@@ -4184,7 +4184,11 @@
           <t>Zazie Productions Publishing</t>
         </is>
       </c>
-      <c r="P21" s="50"/>
+      <c r="P21" s="50" t="inlineStr">
+        <is>
+          <t>01372389230</t>
+        </is>
+      </c>
       <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>BMI</t>
@@ -4314,7 +4318,11 @@
           <t>Zazie Productions Publishing</t>
         </is>
       </c>
-      <c r="P23" s="50"/>
+      <c r="P23" s="50" t="inlineStr">
+        <is>
+          <t>01372389230</t>
+        </is>
+      </c>
       <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>BMI</t>
@@ -4444,7 +4452,11 @@
           <t>Zazie Productions Publishing</t>
         </is>
       </c>
-      <c r="P25" s="50"/>
+      <c r="P25" s="50" t="inlineStr">
+        <is>
+          <t>01372389230</t>
+        </is>
+      </c>
       <c r="Q25" s="9" t="inlineStr">
         <is>
           <t>BMI</t>
@@ -4574,7 +4586,11 @@
           <t>Zazie Productions Publishing</t>
         </is>
       </c>
-      <c r="P27" s="50"/>
+      <c r="P27" s="50" t="inlineStr">
+        <is>
+          <t>01372389230</t>
+        </is>
+      </c>
       <c r="Q27" s="9" t="inlineStr">
         <is>
           <t>BMI</t>
@@ -4704,7 +4720,11 @@
           <t>Zazie Productions Publishing</t>
         </is>
       </c>
-      <c r="P29" s="50"/>
+      <c r="P29" s="50" t="inlineStr">
+        <is>
+          <t>01372389230</t>
+        </is>
+      </c>
       <c r="Q29" s="9" t="inlineStr">
         <is>
           <t>BMI</t>
@@ -4834,7 +4854,11 @@
           <t>Zazie Productions Publishing</t>
         </is>
       </c>
-      <c r="P31" s="50"/>
+      <c r="P31" s="50" t="inlineStr">
+        <is>
+          <t>01372389230</t>
+        </is>
+      </c>
       <c r="Q31" s="9" t="inlineStr">
         <is>
           <t>BMI</t>

</xml_diff>

<commit_message>
Fix Dark Awaits cue sheet workbook compatibility
Rebuild from the untouched 2016 V3-6-5 template using Excel-native shared strings instead of inline strings, refresh formula result caches without changing any formula, and use the template grouped cue-block layout so Seq. numbers cues 1-6 and Total Music Duration is 25:08 rather than double-counted.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Cue_Sheet_The_Dark_Awaits_COMPLETED.xlsx
+++ b/Cue_Sheet_The_Dark_Awaits_COMPLETED.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="302">
   <si>
     <t>Cue Sheet Classification:</t>
   </si>
@@ -895,6 +895,42 @@
   </si>
   <si>
     <t>7/22/2016, 6:41 PM</t>
+  </si>
+  <si>
+    <t>The Dark Awaits</t>
+  </si>
+  <si>
+    <t>Dark Echo Productions</t>
+  </si>
+  <si>
+    <t>Impact Wave Tick Interlude</t>
+  </si>
+  <si>
+    <t>ZAZIE</t>
+  </si>
+  <si>
+    <t>PRODUCTIONS</t>
+  </si>
+  <si>
+    <t>Zazie Productions Publishing</t>
+  </si>
+  <si>
+    <t>01372389230</t>
+  </si>
+  <si>
+    <t>John's Story — Distorted Atmospheric Pad</t>
+  </si>
+  <si>
+    <t>Spirits Still Around</t>
+  </si>
+  <si>
+    <t>Industrial Electronic Interlude</t>
+  </si>
+  <si>
+    <t>Mystic Bell Ambience</t>
+  </si>
+  <si>
+    <t>Family Investigation — Dark Ambience</t>
   </si>
 </sst>
 </file>
@@ -3559,7 +3595,7 @@
     <row r="1" spans="1:18" s="17" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="48" t="str">
         <f>IFERROR(IF($N$4="","Music Cue Sheet Template",IF($N$6="",$N$4,$N$4&amp;", "&amp;$N$6)),"")</f>
-        <v>Music Cue Sheet Template</v>
+        <v>The Dark Awaits</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -3582,7 +3618,7 @@
     <row r="2" spans="1:18" s="17" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="49" t="str">
         <f>IFERROR(IF($A$1="Weekly World of Music, Rock and Roll","Sample Music Cue Sheet",IF($N$4="","",IF(OR($D$4="Revision", $D$4="Revised"),"Revised Music Cue Sheet","Music Cue Sheet"))),"")</f>
-        <v/>
+        <v>Music Cue Sheet</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -3639,10 +3675,8 @@
       <c r="M4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="N4" s="96" t="inlineStr">
-        <is>
-          <t>The Dark Awaits</t>
-        </is>
+      <c r="N4" s="96" t="s">
+        <v>290</v>
       </c>
       <c r="O4" s="96"/>
       <c r="P4" s="96"/>
@@ -3799,10 +3833,8 @@
       <c r="M11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="N11" s="96" t="inlineStr">
-        <is>
-          <t>Dark Echo Productions</t>
-        </is>
+      <c r="N11" s="96" t="s">
+        <v>291</v>
       </c>
       <c r="O11" s="96"/>
       <c r="P11" s="96"/>
@@ -3867,25 +3899,25 @@
       <c r="C14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="5" t="str">
+      <c r="D14" s="5">
         <f>IFERROR(IF(((SUM(J:J)*60)+(SUM(K:K)))=0,"",TRUNC(((SUM(J:J)*60)+(SUM(K:K)))/60)),"")</f>
-        <v/>
+        <v>25</v>
       </c>
       <c r="E14" s="3" t="str">
         <f>IFERROR(IF($D$14="","","min."),"")</f>
-        <v/>
-      </c>
-      <c r="F14" s="5" t="str">
+        <v>min.</v>
+      </c>
+      <c r="F14" s="5">
         <f>IFERROR(IF(((SUM(J:J)*60)+(SUM(K:K)))=0,"",MOD(((SUM(J:J)*60)+(SUM(K:K))),60)),"")</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="G14" s="3" t="str">
         <f>IFERROR(IF($D$14="","","sec."),"")</f>
-        <v/>
+        <v>sec.</v>
       </c>
       <c r="H14" s="8" t="str">
         <f>IFERROR(IF($D$14="","","(auto calc.)"),"")</f>
-        <v/>
+        <v>(auto calc.)</v>
       </c>
       <c r="I14" s="8"/>
       <c r="J14" s="7"/>
@@ -4069,15 +4101,11 @@
         <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
         <v>1</v>
       </c>
-      <c r="B20" s="91" t="inlineStr">
-        <is>
-          <t>Impact Wave Tick Interlude</t>
-        </is>
-      </c>
-      <c r="C20" s="73" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
+      <c r="B20" s="91" t="s">
+        <v>292</v>
+      </c>
+      <c r="C20" s="73" t="s">
+        <v>29</v>
       </c>
       <c r="D20" s="74">
         <v>0</v>
@@ -4097,35 +4125,27 @@
       <c r="I20" s="76">
         <v>35</v>
       </c>
-      <c r="J20" s="74" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
-        <v/>
-      </c>
-      <c r="K20" s="76" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="52" t="inlineStr">
-        <is>
-          <t>Composer</t>
-        </is>
-      </c>
-      <c r="M20" s="73" t="inlineStr">
-        <is>
-          <t>ZAZIE</t>
-        </is>
-      </c>
-      <c r="N20" s="73" t="inlineStr">
-        <is>
-          <t>PRODUCTIONS</t>
-        </is>
+      <c r="J20" s="74">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="76">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>25</v>
+      </c>
+      <c r="M20" s="73" t="s">
+        <v>293</v>
+      </c>
+      <c r="N20" s="73" t="s">
+        <v>294</v>
       </c>
       <c r="O20" s="84"/>
       <c r="P20" s="77"/>
-      <c r="Q20" s="73" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="Q20" s="73" t="s">
+        <v>26</v>
       </c>
       <c r="R20" s="78">
         <v>1</v>
@@ -4136,34 +4156,14 @@
         <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
         <v/>
       </c>
-      <c r="B21" s="92" t="inlineStr">
-        <is>
-          <t>Impact Wave Tick Interlude</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="D21" s="32">
-        <v>0</v>
-      </c>
-      <c r="E21" s="33">
-        <v>2</v>
-      </c>
-      <c r="F21" s="34">
-        <v>32</v>
-      </c>
-      <c r="G21" s="32">
-        <v>0</v>
-      </c>
-      <c r="H21" s="33">
-        <v>2</v>
-      </c>
-      <c r="I21" s="34">
-        <v>35</v>
-      </c>
+      <c r="B21" s="92"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="34"/>
       <c r="J21" s="32" t="str">
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
         <v/>
@@ -4172,46 +4172,34 @@
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
         <v/>
       </c>
-      <c r="L21" s="53" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
+      <c r="L21" s="53" t="s">
+        <v>28</v>
       </c>
       <c r="M21" s="9"/>
       <c r="N21" s="9"/>
-      <c r="O21" s="85" t="inlineStr">
-        <is>
-          <t>Zazie Productions Publishing</t>
-        </is>
-      </c>
-      <c r="P21" s="50" t="inlineStr">
-        <is>
-          <t>01372389230</t>
-        </is>
-      </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="O21" s="85" t="s">
+        <v>295</v>
+      </c>
+      <c r="P21" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q21" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R21" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="81" t="str">
-        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
-        <v/>
-      </c>
-      <c r="B22" s="92" t="inlineStr">
-        <is>
-          <t>John's Story — Distorted Atmospheric Pad</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
+      <c r="A22" s="81">
+        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
+        <v>2</v>
+      </c>
+      <c r="B22" s="92" t="s">
+        <v>297</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>29</v>
       </c>
       <c r="D22" s="32">
         <v>0</v>
@@ -4231,35 +4219,27 @@
       <c r="I22" s="34">
         <v>48</v>
       </c>
-      <c r="J22" s="32" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
-        <v/>
-      </c>
-      <c r="K22" s="34" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="53" t="inlineStr">
-        <is>
-          <t>Composer</t>
-        </is>
-      </c>
-      <c r="M22" s="9" t="inlineStr">
-        <is>
-          <t>ZAZIE</t>
-        </is>
-      </c>
-      <c r="N22" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTIONS</t>
-        </is>
+      <c r="J22" s="32">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
+        <v>0</v>
+      </c>
+      <c r="K22" s="34">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
+        <v>6</v>
+      </c>
+      <c r="L22" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="M22" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>294</v>
       </c>
       <c r="O22" s="85"/>
       <c r="P22" s="50"/>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="Q22" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R22" s="31">
         <v>1</v>
@@ -4270,34 +4250,14 @@
         <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
         <v/>
       </c>
-      <c r="B23" s="92" t="inlineStr">
-        <is>
-          <t>John's Story — Distorted Atmospheric Pad</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="D23" s="32">
-        <v>0</v>
-      </c>
-      <c r="E23" s="33">
-        <v>2</v>
-      </c>
-      <c r="F23" s="34">
-        <v>42</v>
-      </c>
-      <c r="G23" s="32">
-        <v>0</v>
-      </c>
-      <c r="H23" s="33">
-        <v>2</v>
-      </c>
-      <c r="I23" s="34">
-        <v>48</v>
-      </c>
+      <c r="B23" s="92"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="34"/>
       <c r="J23" s="32" t="str">
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
         <v/>
@@ -4306,46 +4266,34 @@
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
         <v/>
       </c>
-      <c r="L23" s="53" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
+      <c r="L23" s="53" t="s">
+        <v>28</v>
       </c>
       <c r="M23" s="9"/>
       <c r="N23" s="9"/>
-      <c r="O23" s="85" t="inlineStr">
-        <is>
-          <t>Zazie Productions Publishing</t>
-        </is>
-      </c>
-      <c r="P23" s="50" t="inlineStr">
-        <is>
-          <t>01372389230</t>
-        </is>
-      </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="O23" s="85" t="s">
+        <v>295</v>
+      </c>
+      <c r="P23" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q23" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R23" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="81" t="str">
-        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
-        <v/>
-      </c>
-      <c r="B24" s="92" t="inlineStr">
-        <is>
-          <t>Spirits Still Around</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
+      <c r="A24" s="81">
+        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
+        <v>3</v>
+      </c>
+      <c r="B24" s="92" t="s">
+        <v>298</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>29</v>
       </c>
       <c r="D24" s="32">
         <v>0</v>
@@ -4365,35 +4313,27 @@
       <c r="I24" s="34">
         <v>25</v>
       </c>
-      <c r="J24" s="32" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
-        <v/>
-      </c>
-      <c r="K24" s="34" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
-        <v/>
-      </c>
-      <c r="L24" s="53" t="inlineStr">
-        <is>
-          <t>Composer</t>
-        </is>
-      </c>
-      <c r="M24" s="9" t="inlineStr">
-        <is>
-          <t>ZAZIE</t>
-        </is>
-      </c>
-      <c r="N24" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTIONS</t>
-        </is>
+      <c r="J24" s="32">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
+        <v>0</v>
+      </c>
+      <c r="K24" s="34">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
+        <v>19</v>
+      </c>
+      <c r="L24" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="M24" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="N24" s="9" t="s">
+        <v>294</v>
       </c>
       <c r="O24" s="85"/>
       <c r="P24" s="50"/>
-      <c r="Q24" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="Q24" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R24" s="31">
         <v>1</v>
@@ -4404,34 +4344,14 @@
         <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
         <v/>
       </c>
-      <c r="B25" s="92" t="inlineStr">
-        <is>
-          <t>Spirits Still Around</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="D25" s="32">
-        <v>0</v>
-      </c>
-      <c r="E25" s="33">
-        <v>4</v>
-      </c>
-      <c r="F25" s="34">
-        <v>6</v>
-      </c>
-      <c r="G25" s="32">
-        <v>0</v>
-      </c>
-      <c r="H25" s="33">
-        <v>4</v>
-      </c>
-      <c r="I25" s="34">
-        <v>25</v>
-      </c>
+      <c r="B25" s="92"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="34"/>
       <c r="J25" s="32" t="str">
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
         <v/>
@@ -4440,46 +4360,34 @@
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
         <v/>
       </c>
-      <c r="L25" s="53" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
+      <c r="L25" s="53" t="s">
+        <v>28</v>
       </c>
       <c r="M25" s="9"/>
       <c r="N25" s="9"/>
-      <c r="O25" s="85" t="inlineStr">
-        <is>
-          <t>Zazie Productions Publishing</t>
-        </is>
-      </c>
-      <c r="P25" s="50" t="inlineStr">
-        <is>
-          <t>01372389230</t>
-        </is>
-      </c>
-      <c r="Q25" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="O25" s="85" t="s">
+        <v>295</v>
+      </c>
+      <c r="P25" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q25" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R25" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="81" t="str">
-        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
-        <v/>
-      </c>
-      <c r="B26" s="92" t="inlineStr">
-        <is>
-          <t>Industrial Electronic Interlude</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
+      <c r="A26" s="81">
+        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
+        <v>4</v>
+      </c>
+      <c r="B26" s="92" t="s">
+        <v>299</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>29</v>
       </c>
       <c r="D26" s="32">
         <v>0</v>
@@ -4499,35 +4407,27 @@
       <c r="I26" s="34">
         <v>49</v>
       </c>
-      <c r="J26" s="32" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
-        <v/>
-      </c>
-      <c r="K26" s="34" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
-        <v/>
-      </c>
-      <c r="L26" s="53" t="inlineStr">
-        <is>
-          <t>Composer</t>
-        </is>
-      </c>
-      <c r="M26" s="9" t="inlineStr">
-        <is>
-          <t>ZAZIE</t>
-        </is>
-      </c>
-      <c r="N26" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTIONS</t>
-        </is>
+      <c r="J26" s="32">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
+        <v>0</v>
+      </c>
+      <c r="K26" s="34">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
+        <v>37</v>
+      </c>
+      <c r="L26" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="M26" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="N26" s="9" t="s">
+        <v>294</v>
       </c>
       <c r="O26" s="85"/>
       <c r="P26" s="50"/>
-      <c r="Q26" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="Q26" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R26" s="31">
         <v>1</v>
@@ -4538,34 +4438,14 @@
         <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
         <v/>
       </c>
-      <c r="B27" s="92" t="inlineStr">
-        <is>
-          <t>Industrial Electronic Interlude</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="D27" s="32">
-        <v>0</v>
-      </c>
-      <c r="E27" s="33">
-        <v>6</v>
-      </c>
-      <c r="F27" s="34">
-        <v>12</v>
-      </c>
-      <c r="G27" s="32">
-        <v>0</v>
-      </c>
-      <c r="H27" s="33">
-        <v>6</v>
-      </c>
-      <c r="I27" s="34">
-        <v>49</v>
-      </c>
+      <c r="B27" s="92"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="34"/>
       <c r="J27" s="32" t="str">
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
         <v/>
@@ -4574,46 +4454,34 @@
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
         <v/>
       </c>
-      <c r="L27" s="53" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
+      <c r="L27" s="53" t="s">
+        <v>28</v>
       </c>
       <c r="M27" s="9"/>
       <c r="N27" s="9"/>
-      <c r="O27" s="85" t="inlineStr">
-        <is>
-          <t>Zazie Productions Publishing</t>
-        </is>
-      </c>
-      <c r="P27" s="50" t="inlineStr">
-        <is>
-          <t>01372389230</t>
-        </is>
-      </c>
-      <c r="Q27" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="O27" s="85" t="s">
+        <v>295</v>
+      </c>
+      <c r="P27" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q27" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R27" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="81" t="str">
-        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
-        <v/>
-      </c>
-      <c r="B28" s="92" t="inlineStr">
-        <is>
-          <t>Mystic Bell Ambience</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
+      <c r="A28" s="81">
+        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
+        <v>5</v>
+      </c>
+      <c r="B28" s="92" t="s">
+        <v>300</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>29</v>
       </c>
       <c r="D28" s="32">
         <v>0</v>
@@ -4633,35 +4501,27 @@
       <c r="I28" s="34">
         <v>0</v>
       </c>
-      <c r="J28" s="32" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
-        <v/>
-      </c>
-      <c r="K28" s="34" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
-        <v/>
-      </c>
-      <c r="L28" s="53" t="inlineStr">
-        <is>
-          <t>Composer</t>
-        </is>
-      </c>
-      <c r="M28" s="9" t="inlineStr">
-        <is>
-          <t>ZAZIE</t>
-        </is>
-      </c>
-      <c r="N28" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTIONS</t>
-        </is>
+      <c r="J28" s="32">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
+        <v>0</v>
+      </c>
+      <c r="K28" s="34">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
+        <v>28</v>
+      </c>
+      <c r="L28" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="M28" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="N28" s="9" t="s">
+        <v>294</v>
       </c>
       <c r="O28" s="85"/>
       <c r="P28" s="50"/>
-      <c r="Q28" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="Q28" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R28" s="31">
         <v>1</v>
@@ -4672,34 +4532,14 @@
         <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
         <v/>
       </c>
-      <c r="B29" s="92" t="inlineStr">
-        <is>
-          <t>Mystic Bell Ambience</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="D29" s="32">
-        <v>0</v>
-      </c>
-      <c r="E29" s="33">
-        <v>7</v>
-      </c>
-      <c r="F29" s="34">
-        <v>32</v>
-      </c>
-      <c r="G29" s="32">
-        <v>0</v>
-      </c>
-      <c r="H29" s="33">
-        <v>8</v>
-      </c>
-      <c r="I29" s="34">
-        <v>0</v>
-      </c>
+      <c r="B29" s="92"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="34"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="34"/>
       <c r="J29" s="32" t="str">
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
         <v/>
@@ -4708,46 +4548,34 @@
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
         <v/>
       </c>
-      <c r="L29" s="53" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
+      <c r="L29" s="53" t="s">
+        <v>28</v>
       </c>
       <c r="M29" s="9"/>
       <c r="N29" s="9"/>
-      <c r="O29" s="85" t="inlineStr">
-        <is>
-          <t>Zazie Productions Publishing</t>
-        </is>
-      </c>
-      <c r="P29" s="50" t="inlineStr">
-        <is>
-          <t>01372389230</t>
-        </is>
-      </c>
-      <c r="Q29" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="O29" s="85" t="s">
+        <v>295</v>
+      </c>
+      <c r="P29" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q29" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R29" s="31">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="81" t="str">
-        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
-        <v/>
-      </c>
-      <c r="B30" s="92" t="inlineStr">
-        <is>
-          <t>Family Investigation — Dark Ambience</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
+      <c r="A30" s="81">
+        <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
+        <v>6</v>
+      </c>
+      <c r="B30" s="92" t="s">
+        <v>301</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>29</v>
       </c>
       <c r="D30" s="32">
         <v>0</v>
@@ -4767,35 +4595,27 @@
       <c r="I30" s="34">
         <v>0</v>
       </c>
-      <c r="J30" s="32" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
-        <v/>
-      </c>
-      <c r="K30" s="34" t="str">
-        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="53" t="inlineStr">
-        <is>
-          <t>Composer</t>
-        </is>
-      </c>
-      <c r="M30" s="9" t="inlineStr">
-        <is>
-          <t>ZAZIE</t>
-        </is>
-      </c>
-      <c r="N30" s="9" t="inlineStr">
-        <is>
-          <t>PRODUCTIONS</t>
-        </is>
+      <c r="J30" s="32">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
+        <v>23</v>
+      </c>
+      <c r="K30" s="34">
+        <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
+        <v>35</v>
+      </c>
+      <c r="L30" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="M30" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="N30" s="9" t="s">
+        <v>294</v>
       </c>
       <c r="O30" s="85"/>
       <c r="P30" s="50"/>
-      <c r="Q30" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="Q30" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R30" s="31">
         <v>1</v>
@@ -4806,34 +4626,14 @@
         <f ca="1">IFERROR(IF((INDIRECT("A"&amp;ROW()-1))="Seq. #",1,IF(ISTEXT(CueDetails2[[#This Row],[Column2]]),COUNTA(INDIRECT("B20"):CueDetails2[[#This Row],[Column2]]),"")),"")</f>
         <v/>
       </c>
-      <c r="B31" s="92" t="inlineStr">
-        <is>
-          <t>Family Investigation — Dark Ambience</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="D31" s="32">
-        <v>0</v>
-      </c>
-      <c r="E31" s="33">
-        <v>14</v>
-      </c>
-      <c r="F31" s="34">
-        <v>25</v>
-      </c>
-      <c r="G31" s="32">
-        <v>0</v>
-      </c>
-      <c r="H31" s="33">
-        <v>38</v>
-      </c>
-      <c r="I31" s="34">
-        <v>0</v>
-      </c>
+      <c r="B31" s="92"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="34"/>
       <c r="J31" s="32" t="str">
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(INT((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]]))/60))),"")</f>
         <v/>
@@ -4842,27 +4642,19 @@
         <f>IFERROR(IF(OR(CueDetails2[[#This Row],[Column6]]="",CueDetails2[[#This Row],[Column9]]=""),"",(MOD(MOD((((CueDetails2[[#This Row],[Column7]]-CueDetails2[[#This Row],[Column4]])*3600)+((CueDetails2[[#This Row],[Column8]]-CueDetails2[[#This Row],[Column5]])*60)+(CueDetails2[[#This Row],[Column9]]-CueDetails2[[#This Row],[Column6]])),3600),60))),"")</f>
         <v/>
       </c>
-      <c r="L31" s="53" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
+      <c r="L31" s="53" t="s">
+        <v>28</v>
       </c>
       <c r="M31" s="9"/>
       <c r="N31" s="9"/>
-      <c r="O31" s="85" t="inlineStr">
-        <is>
-          <t>Zazie Productions Publishing</t>
-        </is>
-      </c>
-      <c r="P31" s="50" t="inlineStr">
-        <is>
-          <t>01372389230</t>
-        </is>
-      </c>
-      <c r="Q31" s="9" t="inlineStr">
-        <is>
-          <t>BMI</t>
-        </is>
+      <c r="O31" s="85" t="s">
+        <v>295</v>
+      </c>
+      <c r="P31" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q31" s="9" t="s">
+        <v>26</v>
       </c>
       <c r="R31" s="31">
         <v>1</v>

</xml_diff>